<commit_message>
use exact original intention registration workbook
</commit_message>
<xml_diff>
--- a/.agents/skills/sourcing-invitation/templates/招标意向征集登记表模板.xlsx
+++ b/.agents/skills/sourcing-invitation/templates/招标意向征集登记表模板.xlsx
@@ -1,3 +1,35 @@
+
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\重庆\2026\26年降本\skill\Original data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <bookViews>
+    <workbookView windowWidth="19200" windowHeight="6420"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+  </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
+</workbook>
+</file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">

</xml_diff>